<commit_message>
Add All Together processing mode (combines survey, undelivered, and dispute)
</commit_message>
<xml_diff>
--- a/1147-Job Done Details-2026-02-03-2026-02-05 (1).xlsx
+++ b/1147-Job Done Details-2026-02-03-2026-02-05 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alquraishi-my.sharepoint.com/personal/abdulrhman_alshehri_starlinks-me_com/Documents/AraBot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_EA710F98B1339FBB9AD4459DA81680C07386E3D7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88DF96A2-07DD-4008-8DB0-32A6DE5FBB00}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_EA710F98B1339FBB9AD4459DA81680C07386E3D7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8E4B987-F049-4E61-8DAC-CFC7112C909A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Job Done Events" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
   <si>
     <t>Event Time</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">Survey for shipment: S0005635403, How was your experience? 5, Recommendation Rate: 10, How is delivery speed? 5, How was package condition? 5, Was the courier's behavior good? 5, Any payment issue? Payment Arabot test, How can we improve? Suggestions arabot test, ||| Shipment Details: status: Delivered, customer name: Starlinks Testing Merchant, service code: ST001, order reference: CTO-3119, customer id reference: , incoterm: , currency: SAR, price: 104, cod value: , cod currency: SAR, consignee name: ali ahmed, consignee city: Riyadh, consignee country: SA, consignee phone: 966509722086, consignee code value: , shipper name: Starlinks Flagship Warehouse, shipper city: riyadh, shipper country: SA, shipper phone: 9668003044433, shipper code value: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Survey for shipment: R0000418068, How was your experience? 5, Recommendation Rate: 10, How is delivery speed? 5, How was package condition? 5, Was the courier's behavior good? 5, Any payment issue? Payment Arabot test, How can we improve? Suggestions arabot test, ||| Shipment Details: status: Delivered, customer name: Starlinks Testing Merchant, service code: ST001, order reference: CTO-3119, customer id reference: , incoterm: , currency: SAR, price: 104, cod value: , cod currency: SAR, consignee name: ali ahmed, consignee city: Riyadh, consignee country: SA, consignee phone: 966509722086, consignee code value: , shipper name: Starlinks Flagship Warehouse, shipper city: riyadh, shipper country: SA, shipper phone: 9668003044433, shipper code value: </t>
   </si>
 </sst>
 </file>
@@ -516,17 +519,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="255" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -543,7 +546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -560,7 +563,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -577,7 +580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -594,7 +597,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -611,7 +614,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -628,7 +631,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -645,7 +648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -662,7 +665,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
@@ -679,7 +682,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
@@ -696,7 +699,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
@@ -711,6 +714,23 @@
       </c>
       <c r="E11" s="2" t="s">
         <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>